<commit_message>
Ask for staff names and positions (who provides, prepares, reviews)
Staff names are welcome; player names remain excluded. Updates labels,
privacy notice, fictional samples and sample exports.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/exports/SAMPLE_submission_1_fictional.xlsx
+++ b/samples/exports/SAMPLE_submission_1_fictional.xlsx
@@ -472,12 +472,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Owner (role or staff name)</t>
+          <t>Owner (name and position)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Reviewer</t>
+          <t>Reviewer (name and position)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Team Doctor</t>
+          <t>Sam Example - Team Doctor</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Sports Scientist</t>
+          <t>Lee Demo - Sports Scientist</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Sports Scientist</t>
+          <t>Lee Demo - Sports Scientist</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Team Doctor</t>
+          <t>Sam Example - Team Doctor</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -806,7 +806,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Team Doctor</t>
+          <t>Sam Example - Team Doctor</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -872,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -888,7 +888,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>AUD-20261022-E73520</t>
+          <t>AUD-20261022-5E91B9</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-22T05:29:28+00:00</t>
+          <t>2026-10-22T05:51:17+00:00</t>
         </is>
       </c>
     </row>
@@ -1002,9 +1002,9 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Head of Medical / Team Doctor: Person (staff name or job title) Team Doctor; Deputy / cover Senior Physiotherapist; Reporting responsibilities Availability status, weekly summary
-Sports scientist: Person (staff name or job title) Sports Scientist; Deputy / cover S&amp;C Coach; Reporting responsibilities GPS, wellness, RPE reports
-Performance / data analyst: Person (staff name or job title) Data Analyst; Reporting responsibilities Dashboards and archive; Notes (incl. detail for 'Other') No deputy defined</t>
+          <t>Head of Medical / Team Doctor: Name Team Doctor; Deputy / cover (name and position) Senior Physiotherapist; Reporting responsibilities Availability status, weekly summary
+Sports scientist: Name Sports Scientist; Deputy / cover (name and position) S&amp;C Coach; Reporting responsibilities GPS, wellness, RPE reports
+Performance / data analyst: Name Data Analyst; Reporting responsibilities Dashboards and archive; Notes (incl. detail for 'Other') No deputy defined</t>
         </is>
       </c>
     </row>
@@ -1067,12 +1067,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Who prepares the daily report? (role)</t>
+          <t>Names and positions of the people who provide it</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Sports scientist</t>
+          <t>Sam Example (Team Doctor), Jo Sample (Physiotherapist), Lee Demo (Sports Scientist)</t>
         </is>
       </c>
     </row>
@@ -1084,68 +1084,68 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Who reviews it before it is shared? (role, or 'nobody')</t>
+          <t>Who prepares the daily report? (name and position)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Team Doctor</t>
+          <t>Lee Demo - Sports Scientist</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>3. Who provides, prepares and reviews the daily report</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Who reviews it before it is shared? (name and position, or 'nobody')</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Sam Example - Team Doctor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>4. Timing</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>When is the information usually entered?</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Before the morning session
 Comment: Physio updates by 08:45.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>4. Timing</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>When should the report be ready?</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Before the staff / coaches' meeting
 Comment: Around 09:30.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>5. The daily dashboard</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Which information should be visible at the top of the daily dashboard? Choose up to three.</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Player availability; Doctor's comment and recommendation; Training modifications</t>
-        </is>
-      </c>
-    </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>What should the daily medical comment communicate?</t>
+          <t>Which information should be visible at the top of the daily dashboard? Choose up to three.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>What happened; What action is recommended; Who should act; By when</t>
+          <t>Player availability; Doctor's comment and recommendation; Training modifications</t>
         </is>
       </c>
     </row>
@@ -1171,12 +1171,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Optional comment on the medical comment format</t>
+          <t>What should the daily medical comment communicate?</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Two lines maximum, action first.</t>
+          <t>What happened; What action is recommended; Who should act; By when</t>
         </is>
       </c>
     </row>
@@ -1188,12 +1188,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>What does the doctor need the dashboard to show?</t>
+          <t>Optional comment on the medical comment format</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Who still has no update today and which follow-ups are due.</t>
+          <t>Two lines maximum, action first.</t>
         </is>
       </c>
     </row>
@@ -1205,12 +1205,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>What does the physical coach need the dashboard to show?</t>
+          <t>What does the doctor need the dashboard to show?</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Who trains modified and the load limits agreed with medical.</t>
+          <t>Who still has no update today and which follow-ups are due.</t>
         </is>
       </c>
     </row>
@@ -1222,29 +1222,29 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>What does the coach need the dashboard to show?</t>
+          <t>What does the physical coach need the dashboard to show?</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Who is available for full training and who is doubtful for the next match.</t>
+          <t>Who trains modified and the load limits agreed with medical.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>6. Counts and definitions</t>
+          <t>5. The daily dashboard</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Which counts or definitions need to be clearer?</t>
+          <t>What does the coach need the dashboard to show?</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Attendance; Availability; AM/PM or repeat entries</t>
+          <t>Who is available for full training and who is doubtful for the next match.</t>
         </is>
       </c>
     </row>
@@ -1256,29 +1256,29 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Briefly, how are these counted today? (optional)</t>
+          <t>Which counts or definitions need to be clearer?</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Attendance is counted per session in one report and per day in another.</t>
+          <t>Attendance; Availability; AM/PM or repeat entries</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>7. Storage and sharing</t>
+          <t>6. Counts and definitions</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Where are the report and its source files stored?</t>
+          <t>Briefly, how are these counted today? (optional)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Google Drive; Email; WhatsApp</t>
+          <t>Attendance is counted per session in one report and per day in another.</t>
         </is>
       </c>
     </row>
@@ -1290,12 +1290,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>How is the report shared?</t>
+          <t>Where are the report and its source files stored?</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Email; WhatsApp</t>
+          <t>Google Drive; Email; WhatsApp</t>
         </is>
       </c>
     </row>
@@ -1307,46 +1307,46 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Optional comment</t>
+          <t>How is the report shared?</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>No single agreed folder yet.</t>
+          <t>Email; WhatsApp</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>8. Biggest improvement</t>
+          <t>7. Storage and sharing</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>What one change would save the department the most time, or improve the report the most?</t>
+          <t>Optional comment</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Enter availability once and have the daily PDF and the weekly summary built from it.</t>
+          <t>No single agreed folder yet.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>9. Prototype feedback</t>
+          <t>8. Biggest improvement</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Who should review the first dashboard prototype?</t>
+          <t>What one change would save the department the most time, or improve the report the most?</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Doctor; Physical coach; Head coach</t>
+          <t>Enter availability once and have the daily PDF and the weekly summary built from it.</t>
         </is>
       </c>
     </row>
@@ -1358,10 +1358,44 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
+          <t>Who should review the first dashboard prototype?</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Doctor; Physical coach; Head coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>9. Prototype feedback</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Names and positions of the reviewers</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Sam Example (Team Doctor), Kim Placeholder (Physical Coach), Head Coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>9. Prototype feedback</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
           <t>Optional comment (e.g. best time for a 20-minute review)</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>After training on a non-match day. Test submission 1 - fictional.</t>
         </is>

</xml_diff>

<commit_message>
Remove the prototype-feedback section
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/exports/SAMPLE_submission_1_fictional.xlsx
+++ b/samples/exports/SAMPLE_submission_1_fictional.xlsx
@@ -872,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -888,7 +888,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>AUD-20261022-5E91B9</t>
+          <t>AUD-20261022-9FB06B</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-22T05:51:17+00:00</t>
+          <t>2026-10-22T08:32:15+00:00</t>
         </is>
       </c>
     </row>
@@ -1347,57 +1347,6 @@
       <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Enter availability once and have the daily PDF and the weekly summary built from it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>9. Prototype feedback</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Who should review the first dashboard prototype?</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Doctor; Physical coach; Head coach</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>9. Prototype feedback</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Names and positions of the reviewers</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Sam Example (Team Doctor), Kim Placeholder (Physical Coach), Head Coach</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>9. Prototype feedback</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Optional comment (e.g. best time for a 20-minute review)</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>After training on a non-match day. Test submission 1 - fictional.</t>
         </is>
       </c>
     </row>

</xml_diff>